<commit_message>
fix cffex switching and stock daily snapshot flow
</commit_message>
<xml_diff>
--- a/情绪指标.xlsx
+++ b/情绪指标.xlsx
@@ -6369,7 +6369,21 @@
       </c>
     </row>
     <row r="312" spans="1:5">
-      <c r="A312" s="1"/>
+      <c r="A312" s="1">
+        <v>46111</v>
+      </c>
+      <c r="B312">
+        <v>23</v>
+      </c>
+      <c r="C312">
+        <v>26</v>
+      </c>
+      <c r="D312">
+        <v>43</v>
+      </c>
+      <c r="E312">
+        <v>45</v>
+      </c>
     </row>
     <row r="313" spans="1:5">
       <c r="A313" s="1"/>

</xml_diff>

<commit_message>
refresh quant index dashboard and emotion sync
</commit_message>
<xml_diff>
--- a/情绪指标.xlsx
+++ b/情绪指标.xlsx
@@ -6386,13 +6386,55 @@
       </c>
     </row>
     <row r="313" spans="1:5">
-      <c r="A313" s="1"/>
+      <c r="A313" s="1">
+        <v>46112</v>
+      </c>
+      <c r="B313">
+        <v>31</v>
+      </c>
+      <c r="C313">
+        <v>19</v>
+      </c>
+      <c r="D313">
+        <v>27</v>
+      </c>
+      <c r="E313">
+        <v>26</v>
+      </c>
     </row>
     <row r="314" spans="1:5">
-      <c r="A314" s="1"/>
+      <c r="A314" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B314">
+        <v>35</v>
+      </c>
+      <c r="C314">
+        <v>31</v>
+      </c>
+      <c r="D314">
+        <v>32</v>
+      </c>
+      <c r="E314">
+        <v>37</v>
+      </c>
     </row>
     <row r="315" spans="1:5">
-      <c r="A315" s="1"/>
+      <c r="A315" s="1">
+        <v>46115</v>
+      </c>
+      <c r="B315">
+        <v>30</v>
+      </c>
+      <c r="C315">
+        <v>20</v>
+      </c>
+      <c r="D315">
+        <v>24</v>
+      </c>
+      <c r="E315">
+        <v>28</v>
+      </c>
     </row>
     <row r="316" spans="1:5">
       <c r="A316" s="1"/>

</xml_diff>

<commit_message>
switch stock temp service to hfq and requeue failed scheduler jobs
</commit_message>
<xml_diff>
--- a/情绪指标.xlsx
+++ b/情绪指标.xlsx
@@ -6437,16 +6437,72 @@
       </c>
     </row>
     <row r="316" spans="1:5">
-      <c r="A316" s="1"/>
+      <c r="A316" s="1">
+        <v>46119</v>
+      </c>
+      <c r="B316">
+        <v>30</v>
+      </c>
+      <c r="C316">
+        <v>21</v>
+      </c>
+      <c r="D316">
+        <v>29</v>
+      </c>
+      <c r="E316">
+        <v>39</v>
+      </c>
     </row>
     <row r="317" spans="1:5">
-      <c r="A317" s="1"/>
+      <c r="A317" s="1">
+        <v>46120</v>
+      </c>
+      <c r="B317">
+        <v>74</v>
+      </c>
+      <c r="C317">
+        <v>74</v>
+      </c>
+      <c r="D317">
+        <v>74</v>
+      </c>
+      <c r="E317">
+        <v>78</v>
+      </c>
     </row>
     <row r="318" spans="1:5">
-      <c r="A318" s="1"/>
+      <c r="A318" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B318">
+        <v>59</v>
+      </c>
+      <c r="C318">
+        <v>62</v>
+      </c>
+      <c r="D318">
+        <v>63</v>
+      </c>
+      <c r="E318">
+        <v>72</v>
+      </c>
     </row>
     <row r="319" spans="1:5">
-      <c r="A319" s="1"/>
+      <c r="A319" s="1">
+        <v>46122</v>
+      </c>
+      <c r="B319">
+        <v>70</v>
+      </c>
+      <c r="C319">
+        <v>78</v>
+      </c>
+      <c r="D319">
+        <v>78</v>
+      </c>
+      <c r="E319">
+        <v>80</v>
+      </c>
     </row>
     <row r="320" spans="1:5">
       <c r="A320" s="1"/>

</xml_diff>

<commit_message>
ship expanded market data pipelines and services
</commit_message>
<xml_diff>
--- a/情绪指标.xlsx
+++ b/情绪指标.xlsx
@@ -1186,7 +1186,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E322"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="11.8181818181818"/>
@@ -6505,13 +6505,157 @@
       </c>
     </row>
     <row r="320" spans="1:5">
-      <c r="A320" s="1"/>
-    </row>
-    <row r="321" spans="1:1">
-      <c r="A321" s="1"/>
-    </row>
-    <row r="322" spans="1:1">
-      <c r="A322" s="1"/>
+      <c r="A320" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B320">
+        <v>69</v>
+      </c>
+      <c r="C320">
+        <v>80</v>
+      </c>
+      <c r="D320">
+        <v>79</v>
+      </c>
+      <c r="E320">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="321" spans="1:5">
+      <c r="A321" s="1">
+        <v>46126</v>
+      </c>
+      <c r="B321">
+        <v>81</v>
+      </c>
+      <c r="C321">
+        <v>87</v>
+      </c>
+      <c r="D321">
+        <v>92</v>
+      </c>
+      <c r="E321">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="322" spans="1:5">
+      <c r="A322" s="1">
+        <v>46127</v>
+      </c>
+      <c r="B322">
+        <v>85</v>
+      </c>
+      <c r="C322">
+        <v>80</v>
+      </c>
+      <c r="D322">
+        <v>82</v>
+      </c>
+      <c r="E322">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="323" spans="1:5">
+      <c r="A323" s="1">
+        <v>46128</v>
+      </c>
+      <c r="B323">
+        <v>82</v>
+      </c>
+      <c r="C323">
+        <v>85</v>
+      </c>
+      <c r="D323">
+        <v>93</v>
+      </c>
+      <c r="E323">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="324" spans="1:5">
+      <c r="A324" s="1">
+        <v>46129</v>
+      </c>
+      <c r="B324">
+        <v>60</v>
+      </c>
+      <c r="C324">
+        <v>74</v>
+      </c>
+      <c r="D324">
+        <v>89</v>
+      </c>
+      <c r="E324">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="325" spans="1:5">
+      <c r="A325" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B325">
+        <v>73</v>
+      </c>
+      <c r="C325">
+        <v>86</v>
+      </c>
+      <c r="D325">
+        <v>93</v>
+      </c>
+      <c r="E325">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="326" spans="1:5">
+      <c r="A326" s="1">
+        <v>46133</v>
+      </c>
+      <c r="B326">
+        <v>66</v>
+      </c>
+      <c r="C326">
+        <v>80</v>
+      </c>
+      <c r="D326">
+        <v>85</v>
+      </c>
+      <c r="E326">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="327" spans="1:5">
+      <c r="A327" s="1">
+        <v>46134</v>
+      </c>
+      <c r="B327">
+        <v>59</v>
+      </c>
+      <c r="C327">
+        <v>87</v>
+      </c>
+      <c r="D327">
+        <v>91</v>
+      </c>
+      <c r="E327">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="328" spans="1:5">
+      <c r="A328" s="1">
+        <v>46135</v>
+      </c>
+      <c r="B328">
+        <v>57</v>
+      </c>
+      <c r="C328">
+        <v>81</v>
+      </c>
+      <c r="D328">
+        <v>76</v>
+      </c>
+      <c r="E328">
+        <v>73</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>